<commit_message>
add new operation in table analyis , count tradeID
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{704412E5-B073-4A46-855B-59BBE6723EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E21ACBAF-DE3E-4DA2-B2BD-603739896001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -16,8 +16,19 @@
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
     <sheet name="data analysis" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -26,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="20">
   <si>
     <t>TradeID</t>
   </si>
@@ -83,6 +94,9 @@
   </si>
   <si>
     <t>XAUUSD</t>
+  </si>
+  <si>
+    <t>TOTAL TRADES</t>
   </si>
 </sst>
 </file>
@@ -3915,9 +3929,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="A1"/>
+  <dimension ref="C5:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5">
+        <f>COUNT(Table1[TradeID])</f>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hnaya ghadi dart add l total profit
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E21ACBAF-DE3E-4DA2-B2BD-603739896001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870B7860-6BB3-44F8-B871-D8833554D109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="21">
   <si>
     <t>TradeID</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>TOTAL TRADES</t>
+  </si>
+  <si>
+    <t>TOTAL PROFIT</t>
   </si>
 </sst>
 </file>
@@ -3929,7 +3932,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:D5"/>
+  <dimension ref="C5:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
@@ -3945,6 +3948,15 @@
         <v>100</v>
       </c>
     </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6">
+        <f>SUM(Table1[Profit])</f>
+        <v>12225</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hnaya zadt avg , max , min
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870B7860-6BB3-44F8-B871-D8833554D109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D133E5-CF8A-4660-97B2-903C6CC8E62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="24">
   <si>
     <t>TradeID</t>
   </si>
@@ -100,6 +100,15 @@
   </si>
   <si>
     <t>TOTAL PROFIT</t>
+  </si>
+  <si>
+    <t>AVERAGE PROFIT</t>
+  </si>
+  <si>
+    <t>MAX PROFIT</t>
+  </si>
+  <si>
+    <t>MIN PROFIT</t>
   </si>
 </sst>
 </file>
@@ -3932,10 +3941,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:D6"/>
+  <dimension ref="C5:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3957,6 +3966,33 @@
         <v>12225</v>
       </c>
     </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7">
+        <f>AVERAGE(Table1[Profit])</f>
+        <v>122.25</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <f>MAX(Table1[Profit])</f>
+        <v>750</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9">
+        <f>MIN(Table1[Profit])</f>
+        <v>-375</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hnaya zadt total win,loss whta win rate total
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D133E5-CF8A-4660-97B2-903C6CC8E62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58C0573-15E9-4B40-8945-127B1F31E818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="27">
   <si>
     <t>TradeID</t>
   </si>
@@ -109,6 +109,15 @@
   </si>
   <si>
     <t>MIN PROFIT</t>
+  </si>
+  <si>
+    <t>TOTAL WIN</t>
+  </si>
+  <si>
+    <t>TOTAL LOSS</t>
+  </si>
+  <si>
+    <t>WIN RATE</t>
   </si>
 </sst>
 </file>
@@ -3941,7 +3950,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:D9"/>
+  <dimension ref="C5:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
@@ -3993,6 +4002,33 @@
         <v>-375</v>
       </c>
     </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10">
+        <f>COUNTIF(Table1[Result],"Win")</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11">
+        <f>COUNTIF(Table1[Result],"Loss")</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12">
+        <f>D10/D5</f>
+        <v>0.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
hnaya zadt pair wkola pair ghadi na7sab lih total trades w profit w avg profit w wins w win rate
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58C0573-15E9-4B40-8945-127B1F31E818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1EA4A8-9750-42C6-A234-5F7B31CB6CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="31">
   <si>
     <t>TradeID</t>
   </si>
@@ -118,6 +118,18 @@
   </si>
   <si>
     <t>WIN RATE</t>
+  </si>
+  <si>
+    <t>PAIR</t>
+  </si>
+  <si>
+    <t>XAUSUD</t>
+  </si>
+  <si>
+    <t>AVG PROFIT</t>
+  </si>
+  <si>
+    <t>WINS</t>
   </si>
 </sst>
 </file>
@@ -260,7 +272,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -440,8 +452,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -556,6 +574,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -601,9 +634,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3950,84 +3985,148 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:D12"/>
+  <dimension ref="C5:H18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
+    <col min="8" max="8" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C5" t="s">
+    <row r="5" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <f>COUNT(Table1[TradeID])</f>
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C6" t="s">
+    <row r="6" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <f>SUM(Table1[Profit])</f>
         <v>12225</v>
       </c>
     </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C7" t="s">
+    <row r="7" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <f>AVERAGE(Table1[Profit])</f>
         <v>122.25</v>
       </c>
     </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C8" t="s">
+    <row r="8" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <f>MAX(Table1[Profit])</f>
         <v>750</v>
       </c>
     </row>
-    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C9" t="s">
+    <row r="9" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <f>MIN(Table1[Profit])</f>
         <v>-375</v>
       </c>
     </row>
-    <row r="10" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
+    <row r="10" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <f>COUNTIF(Table1[Result],"Win")</f>
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
+    <row r="11" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <f>COUNTIF(Table1[Result],"Loss")</f>
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
+    <row r="12" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <f>D10/D5</f>
         <v>0.59</v>
       </c>
+    </row>
+    <row r="14" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
hnaya zadt total trades
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1EA4A8-9750-42C6-A234-5F7B31CB6CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078B4F19-21B6-4A49-BB69-A669832D7B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="30">
   <si>
     <t>TradeID</t>
   </si>
@@ -121,9 +121,6 @@
   </si>
   <si>
     <t>PAIR</t>
-  </si>
-  <si>
-    <t>XAUSUD</t>
   </si>
   <si>
     <t>AVG PROFIT</t>
@@ -4079,10 +4076,10 @@
         <v>20</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>26</v>
@@ -4092,7 +4089,10 @@
       <c r="C15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" s="2">
+        <f>COUNTIF(Table1[Pair],C15)</f>
+        <v>22</v>
+      </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -4102,7 +4102,10 @@
       <c r="C16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="2"/>
+      <c r="D16" s="2">
+        <f>COUNTIF(Table1[Pair],C16)</f>
+        <v>33</v>
+      </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -4110,9 +4113,12 @@
     </row>
     <row r="17" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="2"/>
+        <v>18</v>
+      </c>
+      <c r="D17" s="2">
+        <f>COUNTIF(Table1[Pair],C17)</f>
+        <v>18</v>
+      </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -4122,7 +4128,10 @@
       <c r="C18" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="2"/>
+      <c r="D18" s="2">
+        <f>COUNTIF(Table1[Pair],C18)</f>
+        <v>27</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -4130,5 +4139,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hnaya zadt total profit dyal kola pair.
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078B4F19-21B6-4A49-BB69-A669832D7B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8BE0DE-C532-4E2F-A922-0DE8305B6646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -4093,7 +4093,10 @@
         <f>COUNTIF(Table1[Pair],C15)</f>
         <v>22</v>
       </c>
-      <c r="E15" s="2"/>
+      <c r="E15" s="2">
+        <f>SUMIF(Table1[Pair],C15,Table1[Profit])</f>
+        <v>2900</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -4106,7 +4109,10 @@
         <f>COUNTIF(Table1[Pair],C16)</f>
         <v>33</v>
       </c>
-      <c r="E16" s="2"/>
+      <c r="E16" s="2">
+        <f>SUMIF(Table1[Pair],C16,Table1[Profit])</f>
+        <v>6825</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -4119,7 +4125,10 @@
         <f>COUNTIF(Table1[Pair],C17)</f>
         <v>18</v>
       </c>
-      <c r="E17" s="2"/>
+      <c r="E17" s="2">
+        <f>SUMIF(Table1[Pair],C17,Table1[Profit])</f>
+        <v>575</v>
+      </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -4132,7 +4141,10 @@
         <f>COUNTIF(Table1[Pair],C18)</f>
         <v>27</v>
       </c>
-      <c r="E18" s="2"/>
+      <c r="E18" s="2">
+        <f>SUMIF(Table1[Pair],C18,Table1[Profit])</f>
+        <v>1925</v>
+      </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>

</xml_diff>

<commit_message>
hnaya badalt design dyal table raw data
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8BE0DE-C532-4E2F-A922-0DE8305B6646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3976369-6743-4C05-B223-1E8244A03F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -712,7 +712,7 @@
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
     <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="0"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 

</xml_diff>

<commit_message>
hnata zadr wins trades dyal kona pair
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF99610B-FE5C-46BA-A919-B4A1573DED6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516E851E-B10C-4011-9D10-CB2CECAB704E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -634,12 +634,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3992,7 +3993,7 @@
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.109375" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" customWidth="1"/>
     <col min="8" max="8" width="11.77734375" customWidth="1"/>
   </cols>
@@ -4101,8 +4102,14 @@
         <f>SUMIF(Table1[Pair],C15,Table1[Profit])</f>
         <v>2900</v>
       </c>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="F15" s="5">
+        <f>AVERAGEIF(Table1[Pair],C15,Table1[Profit])</f>
+        <v>131.81818181818181</v>
+      </c>
+      <c r="G15" s="2">
+        <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Win")</f>
+        <v>12</v>
+      </c>
       <c r="H15" s="2"/>
     </row>
     <row r="16" spans="3:8" x14ac:dyDescent="0.3">
@@ -4117,8 +4124,14 @@
         <f>SUMIF(Table1[Pair],C16,Table1[Profit])</f>
         <v>6825</v>
       </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="F16" s="5">
+        <f>AVERAGEIF(Table1[Pair],C16,Table1[Profit])</f>
+        <v>206.81818181818181</v>
+      </c>
+      <c r="G16" s="2">
+        <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Win")</f>
+        <v>23</v>
+      </c>
       <c r="H16" s="2"/>
     </row>
     <row r="17" spans="3:8" x14ac:dyDescent="0.3">
@@ -4133,8 +4146,14 @@
         <f>SUMIF(Table1[Pair],C17,Table1[Profit])</f>
         <v>575</v>
       </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="F17" s="5">
+        <f>AVERAGEIF(Table1[Pair],C17,Table1[Profit])</f>
+        <v>31.944444444444443</v>
+      </c>
+      <c r="G17" s="2">
+        <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Win")</f>
+        <v>8</v>
+      </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" spans="3:8" x14ac:dyDescent="0.3">
@@ -4149,8 +4168,14 @@
         <f>SUMIF(Table1[Pair],C18,Table1[Profit])</f>
         <v>1925</v>
       </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="F18" s="5">
+        <f>AVERAGEIF(Table1[Pair],C18,Table1[Profit])</f>
+        <v>71.296296296296291</v>
+      </c>
+      <c r="G18" s="2">
+        <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Win")</f>
+        <v>16</v>
+      </c>
       <c r="H18" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
I have creat here win rate for every pair
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516E851E-B10C-4011-9D10-CB2CECAB704E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39435E5-25E5-41E7-BD8B-5729D4D8B35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -590,7 +590,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -633,16 +633,18 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -682,6 +684,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Percent" xfId="42" builtinId="5"/>
     <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
@@ -4110,7 +4113,10 @@
         <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Win")</f>
         <v>12</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="6">
+        <f>G15/D15</f>
+        <v>0.54545454545454541</v>
+      </c>
     </row>
     <row r="16" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C16" s="3" t="s">
@@ -4132,7 +4138,10 @@
         <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Win")</f>
         <v>23</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="6">
+        <f t="shared" ref="H16:H18" si="0">G16/D16</f>
+        <v>0.69696969696969702</v>
+      </c>
     </row>
     <row r="17" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
@@ -4154,7 +4163,10 @@
         <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Win")</f>
         <v>8</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="6">
+        <f t="shared" si="0"/>
+        <v>0.44444444444444442</v>
+      </c>
     </row>
     <row r="18" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C18" s="3" t="s">
@@ -4176,7 +4188,10 @@
         <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Win")</f>
         <v>16</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="6">
+        <f t="shared" si="0"/>
+        <v>0.59259259259259256</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
hanya zadt losess wkan khata2 wsa7a7to dyal wins w losess
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39435E5-25E5-41E7-BD8B-5729D4D8B35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8805F338-B126-475B-88E9-F7C32CFAB30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="31">
   <si>
     <t>TradeID</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>WINS</t>
+  </si>
+  <si>
+    <t>LOSSES</t>
   </si>
 </sst>
 </file>
@@ -459,7 +462,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -589,6 +592,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -635,7 +649,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -643,6 +657,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3982,15 +3997,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:H18"/>
+  <dimension ref="C5:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
@@ -3999,9 +4015,10 @@
     <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" customWidth="1"/>
     <col min="8" max="8" width="11.77734375" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -4010,7 +4027,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
@@ -4019,7 +4036,7 @@
         <v>12225</v>
       </c>
     </row>
-    <row r="7" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
@@ -4028,7 +4045,7 @@
         <v>122.25</v>
       </c>
     </row>
-    <row r="8" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
@@ -4037,7 +4054,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="9" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
@@ -4046,7 +4063,7 @@
         <v>-375</v>
       </c>
     </row>
-    <row r="10" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
@@ -4055,7 +4072,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C11" s="3" t="s">
         <v>25</v>
       </c>
@@ -4064,7 +4081,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
@@ -4073,7 +4090,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="14" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C14" s="3" t="s">
         <v>27</v>
       </c>
@@ -4092,108 +4109,133 @@
       <c r="H14" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="15" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="I14" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C15" s="3" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D15" s="2">
         <f>COUNTIF(Table1[Pair],C15)</f>
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E15" s="4">
         <f>SUMIF(Table1[Pair],C15,Table1[Profit])</f>
-        <v>2900</v>
+        <v>575</v>
       </c>
       <c r="F15" s="5">
         <f>AVERAGEIF(Table1[Pair],C15,Table1[Profit])</f>
-        <v>131.81818181818181</v>
+        <v>31.944444444444443</v>
       </c>
       <c r="G15" s="2">
         <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Win")</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H15" s="6">
         <f>G15/D15</f>
-        <v>0.54545454545454541</v>
-      </c>
-    </row>
-    <row r="16" spans="3:8" x14ac:dyDescent="0.3">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="I15" s="2">
+        <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Loss")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C16" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D16" s="2">
         <f>COUNTIF(Table1[Pair],C16)</f>
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E16" s="4">
         <f>SUMIF(Table1[Pair],C16,Table1[Profit])</f>
-        <v>6825</v>
+        <v>1925</v>
       </c>
       <c r="F16" s="5">
         <f>AVERAGEIF(Table1[Pair],C16,Table1[Profit])</f>
-        <v>206.81818181818181</v>
+        <v>71.296296296296291</v>
       </c>
       <c r="G16" s="2">
         <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Win")</f>
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H16" s="6">
-        <f t="shared" ref="H16:H18" si="0">G16/D16</f>
-        <v>0.69696969696969702</v>
-      </c>
-    </row>
-    <row r="17" spans="3:8" x14ac:dyDescent="0.3">
+        <f>G16/D16</f>
+        <v>0.59259259259259256</v>
+      </c>
+      <c r="I16" s="2">
+        <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Loss")</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D17" s="2">
         <f>COUNTIF(Table1[Pair],C17)</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E17" s="4">
         <f>SUMIF(Table1[Pair],C17,Table1[Profit])</f>
-        <v>575</v>
+        <v>2900</v>
       </c>
       <c r="F17" s="5">
         <f>AVERAGEIF(Table1[Pair],C17,Table1[Profit])</f>
-        <v>31.944444444444443</v>
+        <v>131.81818181818181</v>
       </c>
       <c r="G17" s="2">
         <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Win")</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H17" s="6">
-        <f t="shared" si="0"/>
-        <v>0.44444444444444442</v>
-      </c>
-    </row>
-    <row r="18" spans="3:8" x14ac:dyDescent="0.3">
+        <f>G17/D17</f>
+        <v>0.54545454545454541</v>
+      </c>
+      <c r="I17" s="2">
+        <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Loss")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C18" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D18" s="2">
         <f>COUNTIF(Table1[Pair],C18)</f>
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E18" s="4">
         <f>SUMIF(Table1[Pair],C18,Table1[Profit])</f>
-        <v>1925</v>
+        <v>6825</v>
       </c>
       <c r="F18" s="5">
         <f>AVERAGEIF(Table1[Pair],C18,Table1[Profit])</f>
-        <v>71.296296296296291</v>
+        <v>206.81818181818181</v>
       </c>
       <c r="G18" s="2">
         <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Win")</f>
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H18" s="6">
-        <f t="shared" si="0"/>
-        <v>0.59259259259259256</v>
-      </c>
+        <f>G18/D18</f>
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="I18" s="2">
+        <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Loss")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I19" s="7"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:H18">
+    <sortCondition ref="E15:E18"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
hnaya zadt avg profit dyal win dyal kola pair masta9al
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80D0EC4-2003-49EA-B5F9-3E7112CAAF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E09EC08-65B2-404F-A32F-3552016C0A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="33">
   <si>
     <t>TradeID</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>PROFIT CONTRIBUTION</t>
+  </si>
+  <si>
+    <t>AVG WINS</t>
   </si>
 </sst>
 </file>
@@ -652,7 +655,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -660,6 +663,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -4010,7 +4014,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:J19"/>
+  <dimension ref="C5:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
@@ -4021,9 +4025,10 @@
     <col min="8" max="8" width="11.77734375" customWidth="1"/>
     <col min="9" max="9" width="12.6640625" customWidth="1"/>
     <col min="10" max="10" width="19.6640625" customWidth="1"/>
+    <col min="11" max="11" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -4032,7 +4037,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
@@ -4041,7 +4046,7 @@
         <v>12225</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
@@ -4050,7 +4055,7 @@
         <v>122.25</v>
       </c>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
@@ -4059,7 +4064,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
@@ -4068,7 +4073,7 @@
         <v>-375</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
@@ -4077,7 +4082,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C11" s="3" t="s">
         <v>25</v>
       </c>
@@ -4086,7 +4091,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
@@ -4095,7 +4100,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C14" s="3" t="s">
         <v>27</v>
       </c>
@@ -4120,145 +4125,164 @@
       <c r="J14" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="K14" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C15" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D15" s="2">
         <f>COUNTIF(Table1[Pair],C15)</f>
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E15" s="4">
         <f>SUMIF(Table1[Pair],C15,Table1[Profit])</f>
-        <v>575</v>
+        <v>6825</v>
       </c>
       <c r="F15" s="5">
         <f>AVERAGEIF(Table1[Pair],C15,Table1[Profit])</f>
-        <v>31.944444444444443</v>
+        <v>206.81818181818181</v>
       </c>
       <c r="G15" s="2">
         <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Win")</f>
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="H15" s="6">
         <f>G15/D15</f>
-        <v>0.44444444444444442</v>
+        <v>0.69696969696969702</v>
       </c>
       <c r="I15" s="2">
         <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J15" s="8">
+      <c r="J15" s="9">
         <f>E15/$D$6</f>
-        <v>4.7034764826175871E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.3">
+        <v>0.55828220858895705</v>
+      </c>
+      <c r="K15">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Win")</f>
+        <v>346.73913043478262</v>
+      </c>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C16" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D16" s="2">
         <f>COUNTIF(Table1[Pair],C16)</f>
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E16" s="4">
         <f>SUMIF(Table1[Pair],C16,Table1[Profit])</f>
-        <v>1925</v>
+        <v>2900</v>
       </c>
       <c r="F16" s="5">
         <f>AVERAGEIF(Table1[Pair],C16,Table1[Profit])</f>
-        <v>71.296296296296291</v>
+        <v>131.81818181818181</v>
       </c>
       <c r="G16" s="2">
         <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Win")</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H16" s="6">
         <f>G16/D16</f>
-        <v>0.59259259259259256</v>
+        <v>0.54545454545454541</v>
       </c>
       <c r="I16" s="2">
         <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Loss")</f>
-        <v>11</v>
-      </c>
-      <c r="J16" s="8">
-        <f t="shared" ref="J16:J18" si="0">E16/$D$6</f>
-        <v>0.15746421267893659</v>
-      </c>
-    </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="J16" s="9">
+        <f>E16/$D$6</f>
+        <v>0.23721881390593047</v>
+      </c>
+      <c r="K16">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Win")</f>
+        <v>308.33333333333331</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D17" s="2">
         <f>COUNTIF(Table1[Pair],C17)</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E17" s="4">
         <f>SUMIF(Table1[Pair],C17,Table1[Profit])</f>
-        <v>2900</v>
+        <v>1925</v>
       </c>
       <c r="F17" s="5">
         <f>AVERAGEIF(Table1[Pair],C17,Table1[Profit])</f>
-        <v>131.81818181818181</v>
+        <v>71.296296296296291</v>
       </c>
       <c r="G17" s="2">
         <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Win")</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H17" s="6">
         <f>G17/D17</f>
-        <v>0.54545454545454541</v>
+        <v>0.59259259259259256</v>
       </c>
       <c r="I17" s="2">
         <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Loss")</f>
-        <v>10</v>
-      </c>
-      <c r="J17" s="8">
-        <f t="shared" si="0"/>
-        <v>0.23721881390593047</v>
-      </c>
-    </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="J17" s="9">
+        <f>E17/$D$6</f>
+        <v>0.15746421267893659</v>
+      </c>
+      <c r="K17">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Win")</f>
+        <v>246.875</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C18" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D18" s="2">
         <f>COUNTIF(Table1[Pair],C18)</f>
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E18" s="4">
         <f>SUMIF(Table1[Pair],C18,Table1[Profit])</f>
-        <v>6825</v>
+        <v>575</v>
       </c>
       <c r="F18" s="5">
         <f>AVERAGEIF(Table1[Pair],C18,Table1[Profit])</f>
-        <v>206.81818181818181</v>
+        <v>31.944444444444443</v>
       </c>
       <c r="G18" s="2">
         <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Win")</f>
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="H18" s="6">
         <f>G18/D18</f>
-        <v>0.69696969696969702</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="I18" s="2">
         <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J18" s="8">
-        <f t="shared" si="0"/>
-        <v>0.55828220858895705</v>
-      </c>
-    </row>
-    <row r="19" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="I19" s="7"/>
+      <c r="J18" s="9">
+        <f>E18/$D$6</f>
+        <v>4.7034764826175871E-2</v>
+      </c>
+      <c r="K18">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Win")</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="I19" s="8"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:H18">
-    <sortCondition ref="E15:E18"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">
+    <sortCondition descending="1" ref="E14:E18"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hanya zadt avg loss
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E09EC08-65B2-404F-A32F-3552016C0A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93FDCB20-6038-4360-A919-035DC6A1D095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="34">
   <si>
     <t>TradeID</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>AVG WINS</t>
+  </si>
+  <si>
+    <t>AVG PROFIT LOSS</t>
   </si>
 </sst>
 </file>
@@ -655,7 +658,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -663,7 +666,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -4014,7 +4016,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:K19"/>
+  <dimension ref="C5:L19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
@@ -4026,9 +4028,10 @@
     <col min="9" max="9" width="12.6640625" customWidth="1"/>
     <col min="10" max="10" width="19.6640625" customWidth="1"/>
     <col min="11" max="11" width="19.44140625" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -4037,7 +4040,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
@@ -4046,7 +4049,7 @@
         <v>12225</v>
       </c>
     </row>
-    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
@@ -4055,7 +4058,7 @@
         <v>122.25</v>
       </c>
     </row>
-    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
@@ -4064,7 +4067,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="9" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
@@ -4073,7 +4076,7 @@
         <v>-375</v>
       </c>
     </row>
-    <row r="10" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
@@ -4082,7 +4085,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C11" s="3" t="s">
         <v>25</v>
       </c>
@@ -4091,7 +4094,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
@@ -4100,7 +4103,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="14" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C14" s="3" t="s">
         <v>27</v>
       </c>
@@ -4125,11 +4128,14 @@
       <c r="J14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="15" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="L14" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C15" s="3" t="s">
         <v>15</v>
       </c>
@@ -4157,16 +4163,20 @@
         <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="8">
         <f>E15/$D$6</f>
         <v>0.55828220858895705</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="2">
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Win")</f>
         <v>346.73913043478262</v>
       </c>
-    </row>
-    <row r="16" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="L15" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Loss")</f>
+        <v>-115</v>
+      </c>
+    </row>
+    <row r="16" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C16" s="3" t="s">
         <v>9</v>
       </c>
@@ -4194,16 +4204,20 @@
         <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J16" s="9">
+      <c r="J16" s="8">
         <f>E16/$D$6</f>
         <v>0.23721881390593047</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="2">
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Win")</f>
         <v>308.33333333333331</v>
       </c>
-    </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="L16" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Loss")</f>
+        <v>-80</v>
+      </c>
+    </row>
+    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
         <v>13</v>
       </c>
@@ -4231,16 +4245,20 @@
         <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Loss")</f>
         <v>11</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="8">
         <f>E17/$D$6</f>
         <v>0.15746421267893659</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="2">
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Win")</f>
         <v>246.875</v>
       </c>
-    </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="L17" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Loss")</f>
+        <v>-184.09090909090909</v>
+      </c>
+    </row>
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C18" s="3" t="s">
         <v>18</v>
       </c>
@@ -4268,17 +4286,21 @@
         <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="8">
         <f>E18/$D$6</f>
         <v>4.7034764826175871E-2</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="2">
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Win")</f>
         <v>250</v>
       </c>
-    </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="I19" s="8"/>
+      <c r="L18" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Loss")</f>
+        <v>-142.5</v>
+      </c>
+    </row>
+    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="I19" s="7"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">

</xml_diff>

<commit_message>
hnaya zadt avg R
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93FDCB20-6038-4360-A919-035DC6A1D095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6995A31D-E36F-416D-AD1B-75B926F16DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="35">
   <si>
     <t>TradeID</t>
   </si>
@@ -135,10 +135,13 @@
     <t>PROFIT CONTRIBUTION</t>
   </si>
   <si>
-    <t>AVG WINS</t>
+    <t>AVG PROFIT LOSS</t>
   </si>
   <si>
-    <t>AVG PROFIT LOSS</t>
+    <t>AVG PROFIT WINS</t>
+  </si>
+  <si>
+    <t>AVG R</t>
   </si>
 </sst>
 </file>
@@ -658,7 +661,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -666,6 +669,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -4016,7 +4020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:L19"/>
+  <dimension ref="C5:M19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
@@ -4031,7 +4035,7 @@
     <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -4040,7 +4044,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
@@ -4049,7 +4053,7 @@
         <v>12225</v>
       </c>
     </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
@@ -4058,7 +4062,7 @@
         <v>122.25</v>
       </c>
     </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
@@ -4067,7 +4071,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
@@ -4076,7 +4080,7 @@
         <v>-375</v>
       </c>
     </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
@@ -4085,7 +4089,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C11" s="3" t="s">
         <v>25</v>
       </c>
@@ -4094,7 +4098,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
@@ -4103,7 +4107,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="3" t="s">
         <v>27</v>
       </c>
@@ -4129,13 +4133,16 @@
         <v>31</v>
       </c>
       <c r="K14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="M14" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C15" s="3" t="s">
         <v>15</v>
       </c>
@@ -4163,7 +4170,7 @@
         <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J15" s="8">
+      <c r="J15" s="9">
         <f>E15/$D$6</f>
         <v>0.55828220858895705</v>
       </c>
@@ -4175,8 +4182,12 @@
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Loss")</f>
         <v>-115</v>
       </c>
-    </row>
-    <row r="16" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="M15">
+        <f>K15/ABS(L15)</f>
+        <v>3.0151228733459359</v>
+      </c>
+    </row>
+    <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="3" t="s">
         <v>9</v>
       </c>
@@ -4204,7 +4215,7 @@
         <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J16" s="8">
+      <c r="J16" s="9">
         <f>E16/$D$6</f>
         <v>0.23721881390593047</v>
       </c>
@@ -4216,8 +4227,12 @@
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Loss")</f>
         <v>-80</v>
       </c>
-    </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="M16">
+        <f t="shared" ref="M16:M18" si="0">K16/ABS(L16)</f>
+        <v>3.8541666666666665</v>
+      </c>
+    </row>
+    <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
         <v>13</v>
       </c>
@@ -4245,7 +4260,7 @@
         <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Loss")</f>
         <v>11</v>
       </c>
-      <c r="J17" s="8">
+      <c r="J17" s="9">
         <f>E17/$D$6</f>
         <v>0.15746421267893659</v>
       </c>
@@ -4257,8 +4272,12 @@
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Loss")</f>
         <v>-184.09090909090909</v>
       </c>
-    </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="M17">
+        <f t="shared" si="0"/>
+        <v>1.3410493827160495</v>
+      </c>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C18" s="3" t="s">
         <v>18</v>
       </c>
@@ -4286,7 +4305,7 @@
         <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Loss")</f>
         <v>10</v>
       </c>
-      <c r="J18" s="8">
+      <c r="J18" s="9">
         <f>E18/$D$6</f>
         <v>4.7034764826175871E-2</v>
       </c>
@@ -4298,9 +4317,13 @@
         <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Loss")</f>
         <v>-142.5</v>
       </c>
-    </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="I19" s="7"/>
+      <c r="M18">
+        <f t="shared" si="0"/>
+        <v>1.7543859649122806</v>
+      </c>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="I19" s="8"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">

</xml_diff>